<commit_message>
added regression test cases
</commit_message>
<xml_diff>
--- a/testData/E2E_UAT_003_Part_1.xlsx
+++ b/testData/E2E_UAT_003_Part_1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Automation_Project\E2E_Automation\testData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://netapp-my.sharepoint.com/personal/sunilr2_netapp_com/Documents/Desktop/Playwright Python/E2E_Automation/testData/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD9D3438-B479-483A-B481-50BF058FF391}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{BD9D3438-B479-483A-B481-50BF058FF391}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B8CD1758-99B5-40E9-980F-AC6D75745B17}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="21600" windowHeight="13749" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -90,9 +90,6 @@
     <t>Test for Automation</t>
   </si>
   <si>
-    <t>To be Determined Before Qualify Sales Stage</t>
-  </si>
-  <si>
     <t>Direct</t>
   </si>
   <si>
@@ -352,6 +349,9 @@
   </si>
   <si>
     <t>UCPQ</t>
+  </si>
+  <si>
+    <t>To be Determined at Qualify Sales Stage</t>
   </si>
 </sst>
 </file>
@@ -810,7 +810,7 @@
   <sheetData>
     <row r="1" spans="1:58" x14ac:dyDescent="0.4">
       <c r="A1" s="10" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -831,7 +831,7 @@
       <c r="R1" s="10"/>
       <c r="S1" s="10"/>
       <c r="T1" s="10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="U1" s="10"/>
       <c r="V1" s="10"/>
@@ -871,7 +871,7 @@
       <c r="BD1" s="10"/>
       <c r="BE1" s="10"/>
       <c r="BF1" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:58" x14ac:dyDescent="0.4">
@@ -879,7 +879,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C2" s="11"/>
       <c r="D2" s="11"/>
@@ -897,11 +897,11 @@
       <c r="P2" s="11"/>
       <c r="Q2" s="11"/>
       <c r="R2" s="11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="S2" s="11"/>
       <c r="T2" s="11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="U2" s="11"/>
       <c r="V2" s="11"/>
@@ -917,13 +917,13 @@
       <c r="AF2" s="11"/>
       <c r="AG2" s="11"/>
       <c r="AH2" s="11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="AI2" s="11"/>
       <c r="AJ2" s="11"/>
       <c r="AK2" s="11"/>
       <c r="AL2" s="11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="AM2" s="11"/>
       <c r="AN2" s="11"/>
@@ -932,7 +932,7 @@
       <c r="AQ2" s="11"/>
       <c r="AR2" s="11"/>
       <c r="AS2" s="11" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="AT2" s="11"/>
       <c r="AU2" s="11"/>
@@ -940,18 +940,18 @@
       <c r="AW2" s="11"/>
       <c r="AX2" s="11"/>
       <c r="AY2" s="11" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AZ2" s="11"/>
       <c r="BA2" s="11" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="BB2" s="11"/>
       <c r="BC2" s="11"/>
       <c r="BD2" s="11"/>
       <c r="BE2" s="11"/>
       <c r="BF2" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="3" spans="1:58" x14ac:dyDescent="0.4">
@@ -1007,127 +1007,127 @@
         <v>18</v>
       </c>
       <c r="R3" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="S3" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="S3" s="1" t="s">
-        <v>29</v>
-      </c>
       <c r="T3" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="U3" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="U3" s="1" t="s">
+      <c r="V3" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="V3" s="1" t="s">
+      <c r="W3" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="W3" s="1" t="s">
+      <c r="X3" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="X3" s="1" t="s">
+      <c r="Y3" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="Y3" s="1" t="s">
+      <c r="Z3" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="Z3" s="1" t="s">
+      <c r="AA3" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="AA3" s="1" t="s">
+      <c r="AB3" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="AB3" s="1" t="s">
+      <c r="AC3" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="AC3" s="1" t="s">
+      <c r="AD3" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="AD3" s="1" t="s">
+      <c r="AE3" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="AE3" s="1" t="s">
+      <c r="AF3" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="AF3" s="1" t="s">
+      <c r="AG3" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="AG3" s="1" t="s">
-        <v>45</v>
-      </c>
       <c r="AH3" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AI3" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="AJ3" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="AJ3" s="1" t="s">
-        <v>60</v>
-      </c>
       <c r="AK3" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AL3" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="AM3" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="AM3" s="1" t="s">
-        <v>65</v>
-      </c>
       <c r="AN3" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AO3" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="AP3" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="AQ3" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="AQ3" s="1" t="s">
-        <v>73</v>
-      </c>
       <c r="AR3" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="AS3" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="AT3" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="AT3" s="1" t="s">
+      <c r="AU3" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="AU3" s="1" t="s">
+      <c r="AV3" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="AV3" s="1" t="s">
+      <c r="AW3" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="AW3" s="1" t="s">
+      <c r="AX3" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="AX3" s="1" t="s">
+      <c r="AY3" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="AY3" s="1" t="s">
+      <c r="AZ3" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="AZ3" s="1" t="s">
+      <c r="BA3" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="BA3" s="1" t="s">
+      <c r="BB3" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="BB3" s="1" t="s">
+      <c r="BC3" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="BC3" s="1" t="s">
+      <c r="BD3" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="BD3" s="1" t="s">
+      <c r="BE3" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="BE3" s="1" t="s">
+      <c r="BF3" s="1" t="s">
         <v>92</v>
-      </c>
-      <c r="BF3" s="1" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="4" spans="1:58" x14ac:dyDescent="0.4">
@@ -1144,23 +1144,23 @@
         <v>20</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F4" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="G4" s="3" t="s">
         <v>21</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>22</v>
       </c>
       <c r="H4" s="3"/>
       <c r="I4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="J4" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="J4" s="3" t="s">
+      <c r="K4" s="3" t="s">
         <v>24</v>
-      </c>
-      <c r="K4" s="3" t="s">
-        <v>25</v>
       </c>
       <c r="L4" s="3"/>
       <c r="M4" s="3"/>
@@ -1169,127 +1169,127 @@
       <c r="P4" s="3"/>
       <c r="Q4" s="3"/>
       <c r="R4" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="S4" s="4">
         <v>1000</v>
       </c>
       <c r="T4" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="U4" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="U4" s="3" t="s">
+      <c r="V4" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="V4" s="3" t="s">
+      <c r="W4" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="W4" s="3" t="s">
+      <c r="X4" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="X4" s="3" t="s">
+      <c r="Y4" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="Y4" s="3" t="s">
+      <c r="Z4" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="Z4" s="3" t="s">
+      <c r="AA4" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="AB4" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="AC4" s="3" t="s">
         <v>52</v>
-      </c>
-      <c r="AA4" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="AB4" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="AC4" s="3" t="s">
-        <v>53</v>
       </c>
       <c r="AD4" s="4">
         <v>6</v>
       </c>
       <c r="AE4" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="AF4" s="5">
         <v>4</v>
       </c>
       <c r="AG4" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AH4" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="AH4" s="3" t="s">
-        <v>56</v>
-      </c>
       <c r="AI4" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="AJ4" s="4">
         <v>1</v>
       </c>
       <c r="AK4" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="AL4" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="AM4" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="AN4" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="AN4" s="3" t="s">
-        <v>67</v>
-      </c>
       <c r="AO4" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AP4" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="AQ4" s="4">
         <v>6</v>
       </c>
       <c r="AR4" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="AS4" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="AT4" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="AT4" s="3" t="s">
-        <v>103</v>
-      </c>
       <c r="AU4" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="AV4" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="AV4" s="3" t="s">
-        <v>103</v>
-      </c>
       <c r="AW4" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="AX4" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="AX4" s="3" t="s">
+      <c r="AY4" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="AY4" s="3" t="s">
+      <c r="AZ4" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="BA4" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="AZ4" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="BA4" s="7" t="s">
+      <c r="BB4" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="BC4" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="BB4" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="BC4" s="3" t="s">
+      <c r="BD4" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="BD4" s="3" t="s">
+      <c r="BE4" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="BE4" s="3" t="s">
+      <c r="BF4" s="7" t="s">
         <v>100</v>
-      </c>
-      <c r="BF4" s="7" t="s">
-        <v>101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>